<commit_message>
testing missing rows in stages
</commit_message>
<xml_diff>
--- a/HTTP_1/TC1/Detail.xlsx
+++ b/HTTP_1/TC1/Detail.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\HTTP_PE_Contruct\TC1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\auto-grading\HTTP_1\TC1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA176A6B-9831-4383-A60F-F561907F3CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BA2B170-0C20-4B09-8157-7418F082F6A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
   <si>
     <t>Stage</t>
   </si>
@@ -146,64 +146,6 @@
   </si>
   <si>
     <t>Server responding (SYN-ACK)</t>
-  </si>
-  <si>
-    <t>ACK</t>
-  </si>
-  <si>
-    <t>Connection established</t>
-  </si>
-  <si>
-    <t>HTTP Request</t>
-  </si>
-  <si>
-    <t>PSH, ACK</t>
-  </si>
-  <si>
-    <t>Data transfer in progress</t>
-  </si>
-  <si>
-    <t>/books/1</t>
-  </si>
-  <si>
-    <t>localhost:8000</t>
-  </si>
-  <si>
-    <t>GET</t>
-  </si>
-  <si>
-    <t>HTTP/1.1</t>
-  </si>
-  <si>
-    <t>Host: localhost:8000</t>
-  </si>
-  <si>
-    <t>2025-11-25 04:05:46</t>
-  </si>
-  <si>
-    <t>HTTP Response</t>
-  </si>
-  <si>
-    <t>200 OK</t>
-  </si>
-  <si>
-    <t>Content-Length: 268; Content-Type: application/json; Server: Microsoft-HTTPAPI/2.0; Date: Tue, 25 Nov 2025 04:05:46 GMT</t>
-  </si>
-  <si>
-    <t>[
-  {
-    "BookId": 1,
-    "Title": "Harry Potter and the Philosopher\u0027s Stone",
-    "PublicationYear": 1997,
-    "GenreName": "Fantasy"
-  },
-  {
-    "BookId": 3,
-    "Title": "The Hobbit",
-    "PublicationYear": 1937,
-    "GenreName": "Fantasy"
-  }
-]</t>
   </si>
 </sst>
 </file>
@@ -854,28 +796,14 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>38</v>
-      </c>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
       <c r="J4" s="3"/>
@@ -883,83 +811,35 @@
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
-      <c r="O4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>3</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>44</v>
-      </c>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
       <c r="K5" s="3"/>
-      <c r="L5" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>3</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -967,79 +847,35 @@
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
       <c r="N6" s="3"/>
-      <c r="O6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="409.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>41</v>
-      </c>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
       <c r="J7" s="3"/>
-      <c r="K7" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="N7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>3</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>38</v>
-      </c>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
       <c r="J8" s="3"/>
@@ -1047,12 +883,8 @@
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
       <c r="N8" s="3"/>
-      <c r="O8" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>34</v>
-      </c>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>